<commit_message>
Done with current fitting
</commit_message>
<xml_diff>
--- a/BeatnotePostHotCellF1=4/Jul15,2026/Fit_ResultJul15.xlsx
+++ b/BeatnotePostHotCellF1=4/Jul15,2026/Fit_ResultJul15.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diego\git\6s7p\BeatnotePostHotCell\Jul15,2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Wolfwalker\Documents\git\6s7p\BeatnotePostHotCellF1=4\Jul15,2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4D4E329-BDF7-4DD3-B368-4B7F23B456D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CB15DB4-E605-46C6-BD9D-4124D6BB4DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{D9E101C5-8284-4B59-8B1C-2AD2D5F2FDD3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{D9E101C5-8284-4B59-8B1C-2AD2D5F2FDD3}"/>
   </bookViews>
   <sheets>
     <sheet name="894" sheetId="2" r:id="rId1"/>
@@ -150,7 +150,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -522,9 +522,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40C5617D-2BBC-4C21-ADC4-3687FEC8C6E3}">
   <dimension ref="A1:V33"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:22">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -559,7 +559,7 @@
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
     </row>
-    <row r="2" spans="1:22" ht="42.75">
+    <row r="2" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -592,7 +592,7 @@
       <c r="S2" s="1"/>
       <c r="T2" s="1"/>
     </row>
-    <row r="3" spans="1:22" ht="42.75">
+    <row r="3" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -619,7 +619,7 @@
       <c r="U3" s="1"/>
       <c r="V3" s="1"/>
     </row>
-    <row r="4" spans="1:22" ht="42.75">
+    <row r="4" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -644,7 +644,7 @@
       <c r="H4" s="1"/>
       <c r="T4" s="1"/>
     </row>
-    <row r="5" spans="1:22" ht="42.75">
+    <row r="5" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -669,7 +669,7 @@
       <c r="H5" s="1"/>
       <c r="T5" s="1"/>
     </row>
-    <row r="6" spans="1:22" ht="42.75">
+    <row r="6" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -694,7 +694,7 @@
       <c r="H6" s="1"/>
       <c r="T6" s="1"/>
     </row>
-    <row r="7" spans="1:22" ht="42.75">
+    <row r="7" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
@@ -719,7 +719,7 @@
       <c r="H7" s="1"/>
       <c r="T7" s="1"/>
     </row>
-    <row r="8" spans="1:22" ht="42.75">
+    <row r="8" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
@@ -744,7 +744,7 @@
       <c r="H8" s="1"/>
       <c r="T8" s="1"/>
     </row>
-    <row r="9" spans="1:22" ht="42.75">
+    <row r="9" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
@@ -769,7 +769,7 @@
       <c r="H9" s="1"/>
       <c r="T9" s="1"/>
     </row>
-    <row r="10" spans="1:22" ht="42.75">
+    <row r="10" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
@@ -794,7 +794,7 @@
       <c r="H10" s="1"/>
       <c r="T10" s="1"/>
     </row>
-    <row r="11" spans="1:22" ht="42.75">
+    <row r="11" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
@@ -819,7 +819,7 @@
       <c r="H11" s="1"/>
       <c r="T11" s="1"/>
     </row>
-    <row r="12" spans="1:22" ht="42.75">
+    <row r="12" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
@@ -844,7 +844,7 @@
       <c r="H12" s="1"/>
       <c r="T12" s="1"/>
     </row>
-    <row r="13" spans="1:22" ht="42.75">
+    <row r="13" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>22</v>
       </c>
@@ -869,7 +869,7 @@
       <c r="H13" s="1"/>
       <c r="T13" s="1"/>
     </row>
-    <row r="14" spans="1:22" ht="42.75">
+    <row r="14" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>23</v>
       </c>
@@ -894,7 +894,7 @@
       <c r="H14" s="1"/>
       <c r="T14" s="1"/>
     </row>
-    <row r="15" spans="1:22" ht="42.75">
+    <row r="15" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>24</v>
       </c>
@@ -919,7 +919,7 @@
       <c r="H15" s="1"/>
       <c r="T15" s="1"/>
     </row>
-    <row r="16" spans="1:22" ht="42.75">
+    <row r="16" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>25</v>
       </c>
@@ -944,7 +944,7 @@
       <c r="H16" s="1"/>
       <c r="T16" s="1"/>
     </row>
-    <row r="17" spans="1:20" ht="42.75">
+    <row r="17" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>26</v>
       </c>
@@ -969,7 +969,7 @@
       <c r="H17" s="1"/>
       <c r="T17" s="1"/>
     </row>
-    <row r="18" spans="1:20" ht="42.75">
+    <row r="18" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>27</v>
       </c>
@@ -994,7 +994,7 @@
       <c r="H18" s="1"/>
       <c r="T18" s="1"/>
     </row>
-    <row r="19" spans="1:20" ht="42.75">
+    <row r="19" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>28</v>
       </c>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="H19" s="1"/>
     </row>
-    <row r="20" spans="1:20" ht="42.75">
+    <row r="20" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>29</v>
       </c>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="H20" s="1"/>
     </row>
-    <row r="21" spans="1:20" ht="42.75">
+    <row r="21" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>30</v>
       </c>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="H21" s="1"/>
     </row>
-    <row r="22" spans="1:20" ht="42.75">
+    <row r="22" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>31</v>
       </c>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="H22" s="1"/>
     </row>
-    <row r="23" spans="1:20" ht="42.75">
+    <row r="23" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>32</v>
       </c>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="H23" s="1"/>
     </row>
-    <row r="24" spans="1:20" ht="42.75">
+    <row r="24" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>33</v>
       </c>
@@ -1138,7 +1138,7 @@
       </c>
       <c r="H24" s="1"/>
     </row>
-    <row r="25" spans="1:20" ht="42.75">
+    <row r="25" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>34</v>
       </c>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="H25" s="1"/>
     </row>
-    <row r="26" spans="1:20">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -1172,7 +1172,7 @@
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
     </row>
-    <row r="27" spans="1:20">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -1182,7 +1182,7 @@
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
     </row>
-    <row r="28" spans="1:20">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -1192,7 +1192,7 @@
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
     </row>
-    <row r="29" spans="1:20">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -1202,7 +1202,7 @@
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
     </row>
-    <row r="30" spans="1:20">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -1212,7 +1212,7 @@
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
     </row>
-    <row r="31" spans="1:20">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -1222,7 +1222,7 @@
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
     </row>
-    <row r="32" spans="1:20">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -1232,7 +1232,7 @@
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
     </row>
-    <row r="33" spans="1:7">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -1249,12 +1249,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{011646E0-737D-49FA-A2CA-7848F848076B}">
   <dimension ref="A1:T34"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="4" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1290,12 +1290,12 @@
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
     </row>
-    <row r="2" spans="1:20" ht="42.75">
+    <row r="2" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B2" s="1">
-        <v>0.10788210556906901</v>
+        <v>8.4020421663362793E-2</v>
       </c>
       <c r="C2" s="1">
         <v>1.62513102048731</v>
@@ -1307,13 +1307,13 @@
         <v>1.3680746389313099E-4</v>
       </c>
       <c r="F2" s="1">
-        <v>2.8958485334552302</v>
+        <v>2.8346262897436501</v>
       </c>
       <c r="G2" s="1">
-        <v>40.2640038402795</v>
+        <v>40.223160571235198</v>
       </c>
       <c r="H2" s="1">
-        <v>6.2030213263042496E-4</v>
+        <v>5.8690630075372205E-4</v>
       </c>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
@@ -1325,12 +1325,12 @@
       <c r="S2" s="1"/>
       <c r="T2" s="1"/>
     </row>
-    <row r="3" spans="1:20" ht="42.75">
+    <row r="3" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B3" s="1">
-        <v>0.107767689685955</v>
+        <v>8.3856539409502107E-2</v>
       </c>
       <c r="C3" s="1">
         <v>1.6249358237031899</v>
@@ -1342,22 +1342,22 @@
         <v>1.08117832211795E-4</v>
       </c>
       <c r="F3" s="1">
-        <v>2.8952338587180302</v>
+        <v>2.8340158389465899</v>
       </c>
       <c r="G3" s="1">
-        <v>41.1893708618544</v>
+        <v>40.1914120152001</v>
       </c>
       <c r="H3" s="1">
-        <v>7.5220889368145E-4</v>
+        <v>5.9297948114260903E-4</v>
       </c>
       <c r="L3" s="1"/>
     </row>
-    <row r="4" spans="1:20" ht="42.75">
+    <row r="4" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B4" s="1">
-        <v>0.1085661885666</v>
+        <v>8.4441497497705006E-2</v>
       </c>
       <c r="C4" s="1">
         <v>1.6245069740189599</v>
@@ -1369,21 +1369,21 @@
         <v>7.9107965907056595E-5</v>
       </c>
       <c r="F4" s="1">
-        <v>3.1065289929962199</v>
+        <v>3.04532794030809</v>
       </c>
       <c r="G4" s="1">
-        <v>42.1504244181559</v>
+        <v>41.467682752163498</v>
       </c>
       <c r="H4" s="1">
-        <v>1.14168097877784E-3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20" ht="42.75">
+        <v>5.8817665654652997E-4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B5" s="1">
-        <v>0.107813849166461</v>
+        <v>8.3922207540377103E-2</v>
       </c>
       <c r="C5" s="1">
         <v>1.62601974137552</v>
@@ -1395,21 +1395,21 @@
         <v>1.1775189892077999E-4</v>
       </c>
       <c r="F5" s="1">
-        <v>2.6475533105943301</v>
+        <v>2.5863440222072098</v>
       </c>
       <c r="G5" s="1">
-        <v>41.629912012557199</v>
+        <v>40.200228931305404</v>
       </c>
       <c r="H5" s="1">
-        <v>5.80759086709055E-4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20" ht="42.75">
+        <v>8.1706825247685898E-4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B6" s="1">
-        <v>0.10768118552928301</v>
+        <v>8.3819979532311101E-2</v>
       </c>
       <c r="C6" s="1">
         <v>1.6255265789138</v>
@@ -1421,21 +1421,21 @@
         <v>4.28245980683294E-5</v>
       </c>
       <c r="F6" s="1">
-        <v>2.64429438218446</v>
+        <v>2.5830889445407599</v>
       </c>
       <c r="G6" s="1">
-        <v>41.142942912964003</v>
+        <v>40.5432642988008</v>
       </c>
       <c r="H6" s="1">
-        <v>7.5220751031553697E-4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" ht="42.75">
+        <v>6.3106651764923305E-4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B7" s="1">
-        <v>0.10798815957236201</v>
+        <v>8.4065913892834104E-2</v>
       </c>
       <c r="C7" s="1">
         <v>1.6255816549345901</v>
@@ -1447,21 +1447,21 @@
         <v>3.1242256552500798E-5</v>
       </c>
       <c r="F7" s="1">
-        <v>2.6457065423386599</v>
+        <v>2.58451748234826</v>
       </c>
       <c r="G7" s="1">
-        <v>41.855263179843597</v>
+        <v>41.117922419260097</v>
       </c>
       <c r="H7" s="1">
-        <v>7.5608917501536498E-4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" ht="42.75">
+        <v>7.5220882825701297E-4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B8" s="1">
-        <v>0.10796561723725399</v>
+        <v>8.4094869806041694E-2</v>
       </c>
       <c r="C8" s="1">
         <v>1.62551201595841</v>
@@ -1473,21 +1473,21 @@
         <v>9.8714506108644594E-6</v>
       </c>
       <c r="F8" s="1">
-        <v>2.6461111796097501</v>
+        <v>2.58490172326833</v>
       </c>
       <c r="G8" s="1">
-        <v>41.107368392771399</v>
+        <v>41.107364927779997</v>
       </c>
       <c r="H8" s="1">
-        <v>7.5220762983235496E-4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" ht="42.75">
+        <v>7.5220749611244698E-4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B9" s="1">
-        <v>0.107310696139959</v>
+        <v>8.3498425913598198E-2</v>
       </c>
       <c r="C9" s="1">
         <v>1.6256390914637899</v>
@@ -1499,21 +1499,21 @@
         <v>2.3642404363777402E-5</v>
       </c>
       <c r="F9" s="1">
-        <v>2.6064209221097299</v>
+        <v>2.54523081391469</v>
       </c>
       <c r="G9" s="1">
-        <v>41.0507646787092</v>
+        <v>40.054037104655997</v>
       </c>
       <c r="H9" s="1">
-        <v>7.5220672203154203E-4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:20" ht="42.75">
+        <v>5.8124965138899802E-4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B10" s="1">
-        <v>0.107235378128852</v>
+        <v>8.3501392552088799E-2</v>
       </c>
       <c r="C10" s="1">
         <v>1.6253041511213999</v>
@@ -1525,21 +1525,21 @@
         <v>4.5526386459295999E-5</v>
       </c>
       <c r="F10" s="1">
-        <v>2.6453095573124399</v>
+        <v>2.5841176459942199</v>
       </c>
       <c r="G10" s="1">
-        <v>41.7438006770927</v>
+        <v>41.050884174064599</v>
       </c>
       <c r="H10" s="1">
-        <v>6.6053362679605195E-4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" ht="42.75">
+        <v>7.52209517240325E-4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B11" s="1">
-        <v>0.107380313151722</v>
+        <v>8.3538886283743397E-2</v>
       </c>
       <c r="C11" s="1">
         <v>1.6257007213976</v>
@@ -1551,21 +1551,21 @@
         <v>4.6015841407316202E-5</v>
       </c>
       <c r="F11" s="1">
-        <v>2.6449212985361199</v>
+        <v>2.5837187892525599</v>
       </c>
       <c r="G11" s="1">
-        <v>41.828803030264503</v>
+        <v>40.360374717657798</v>
       </c>
       <c r="H11" s="1">
-        <v>7.0223059968995501E-4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:20" ht="42.75">
+        <v>6.1569350803761095E-4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B12" s="1">
-        <v>0.107499657333732</v>
+        <v>8.3653316711863296E-2</v>
       </c>
       <c r="C12" s="1">
         <v>1.62546584925452</v>
@@ -1577,21 +1577,21 @@
         <v>4.0531543291343298E-5</v>
       </c>
       <c r="F12" s="1">
-        <v>2.6460147362636</v>
+        <v>2.58480731567801</v>
       </c>
       <c r="G12" s="1">
-        <v>41.049688076482802</v>
+        <v>40.140341586243999</v>
       </c>
       <c r="H12" s="1">
-        <v>7.5220981695020301E-4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:20" ht="42.75">
+        <v>5.8350097360163999E-4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B13" s="1">
-        <v>0.107395325995434</v>
+        <v>8.36218907831483E-2</v>
       </c>
       <c r="C13" s="1">
         <v>1.6252953547019899</v>
@@ -1603,21 +1603,21 @@
         <v>1.31936681692726E-5</v>
       </c>
       <c r="F13" s="1">
-        <v>2.6447335173711202</v>
+        <v>2.5835562626950299</v>
       </c>
       <c r="G13" s="1">
-        <v>41.886883193947803</v>
+        <v>41.9694381982953</v>
       </c>
       <c r="H13" s="1">
-        <v>8.93619892199126E-4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:20" ht="42.75">
+        <v>6.4007120018308797E-4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B14" s="1">
-        <v>0.107617315330632</v>
+        <v>8.3768728051409405E-2</v>
       </c>
       <c r="C14" s="1">
         <v>1.6245182577871</v>
@@ -1629,21 +1629,21 @@
         <v>3.6398474751521E-5</v>
       </c>
       <c r="F14" s="1">
-        <v>2.64605084777862</v>
+        <v>2.5848254924751899</v>
       </c>
       <c r="G14" s="1">
-        <v>41.135540286681099</v>
+        <v>39.996692696009397</v>
       </c>
       <c r="H14" s="1">
-        <v>5.7956493201096295E-4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:20" ht="42.75">
+        <v>6.3943024656527305E-4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B15" s="1">
-        <v>0.107631821742582</v>
+        <v>8.3798815283381206E-2</v>
       </c>
       <c r="C15" s="1">
         <v>1.62302582925359</v>
@@ -1655,21 +1655,21 @@
         <v>3.2978249826565998E-5</v>
       </c>
       <c r="F15" s="1">
-        <v>2.64581349028653</v>
+        <v>2.5846080451701599</v>
       </c>
       <c r="G15" s="1">
-        <v>40.656111454703101</v>
+        <v>39.979091249866499</v>
       </c>
       <c r="H15" s="1">
-        <v>5.9434649936729203E-4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:20" ht="42.75">
+        <v>6.0835060723521905E-4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B16" s="1">
-        <v>0.107773221003444</v>
+        <v>8.37952938220691E-2</v>
       </c>
       <c r="C16" s="1">
         <v>1.6228942675268201</v>
@@ -1681,21 +1681,21 @@
         <v>8.8334409501128998E-6</v>
       </c>
       <c r="F16" s="1">
-        <v>2.6444357745403302</v>
+        <v>2.5832236291458499</v>
       </c>
       <c r="G16" s="1">
-        <v>41.679491453630597</v>
+        <v>40.094069489653101</v>
       </c>
       <c r="H16" s="1">
-        <v>1.1315730983676401E-3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="42.75">
+        <v>7.6147635156313296E-4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B17" s="1">
-        <v>0.108054680115061</v>
+        <v>8.4084000178888202E-2</v>
       </c>
       <c r="C17" s="1">
         <v>1.62367779985697</v>
@@ -1707,21 +1707,21 @@
         <v>-1.03487801371989E-5</v>
       </c>
       <c r="F17" s="1">
-        <v>2.3956198737559999</v>
+        <v>2.3344052232530501</v>
       </c>
       <c r="G17" s="1">
-        <v>41.611966167156297</v>
+        <v>40.455567406961798</v>
       </c>
       <c r="H17" s="1">
-        <v>6.4948537660913395E-4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="42.75">
+        <v>5.8326986875078201E-4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B18" s="1">
-        <v>0.108470442647848</v>
+        <v>8.4478909636109295E-2</v>
       </c>
       <c r="C18" s="1">
         <v>1.6238014848100799</v>
@@ -1733,21 +1733,21 @@
         <v>-4.7389435126653299E-5</v>
       </c>
       <c r="F18" s="1">
-        <v>2.6467168650612498</v>
+        <v>2.58553271514038</v>
       </c>
       <c r="G18" s="1">
-        <v>41.896587987747097</v>
+        <v>41.896627929150497</v>
       </c>
       <c r="H18" s="1">
-        <v>1.1320425640195099E-3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="42.75">
+        <v>1.07259539268625E-3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B19" s="1">
-        <v>0.108306765636387</v>
+        <v>8.4376066440544406E-2</v>
       </c>
       <c r="C19" s="1">
         <v>1.6234064574068501</v>
@@ -1759,21 +1759,21 @@
         <v>1.1224088142636001E-6</v>
       </c>
       <c r="F19" s="1">
-        <v>2.6464563920608799</v>
+        <v>2.5852526000441198</v>
       </c>
       <c r="G19" s="1">
-        <v>40.901289089830797</v>
+        <v>40.109903559280802</v>
       </c>
       <c r="H19" s="1">
-        <v>7.5220828627167301E-4</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="42.75">
+        <v>1.1531731021658801E-3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B20" s="1">
-        <v>0.10817681982411</v>
+        <v>8.42642456111901E-2</v>
       </c>
       <c r="C20" s="1">
         <v>1.62377726407787</v>
@@ -1785,21 +1785,21 @@
         <v>-2.2156345038941499E-5</v>
       </c>
       <c r="F20" s="1">
-        <v>2.6442350670036201</v>
+        <v>2.5830153614124902</v>
       </c>
       <c r="G20" s="1">
-        <v>40.889269163850102</v>
+        <v>40.889262717686499</v>
       </c>
       <c r="H20" s="1">
-        <v>7.52206885313714E-4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="42.75">
+        <v>7.5220743186441301E-4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B21" s="1">
-        <v>0.107850584510117</v>
+        <v>8.3954508319290494E-2</v>
       </c>
       <c r="C21" s="1">
         <v>1.6240565782905501</v>
@@ -1811,21 +1811,21 @@
         <v>1.20449041040017E-5</v>
       </c>
       <c r="F21" s="1">
-        <v>2.6478975169047199</v>
+        <v>2.58664415720675</v>
       </c>
       <c r="G21" s="1">
-        <v>40.593800496347903</v>
+        <v>39.897409359373803</v>
       </c>
       <c r="H21" s="1">
-        <v>6.6843524962969603E-4</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="42.75">
+        <v>5.8524979762537995E-4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B22" s="1">
-        <v>0.108220094487482</v>
+        <v>8.4241621326531999E-2</v>
       </c>
       <c r="C22" s="1">
         <v>1.6239961691654601</v>
@@ -1837,21 +1837,21 @@
         <v>-1.09974660525283E-6</v>
       </c>
       <c r="F22" s="1">
-        <v>2.6461886383531898</v>
+        <v>2.5849751855913401</v>
       </c>
       <c r="G22" s="1">
-        <v>40.925882036729199</v>
+        <v>39.925563028969798</v>
       </c>
       <c r="H22" s="1">
-        <v>7.5220948797134095E-4</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="42.75">
+        <v>7.9818266589595896E-4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B23" s="1">
-        <v>0.107772509976481</v>
+        <v>8.39433811384213E-2</v>
       </c>
       <c r="C23" s="1">
         <v>1.6251146986004401</v>
@@ -1863,21 +1863,21 @@
         <v>1.0348276531822001E-5</v>
       </c>
       <c r="F23" s="1">
-        <v>2.3562108726532398</v>
+        <v>2.2950163054263402</v>
       </c>
       <c r="G23" s="1">
-        <v>39.922580179559702</v>
+        <v>39.922648811042301</v>
       </c>
       <c r="H23" s="1">
-        <v>5.7871129073961899E-4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="42.75">
+        <v>6.2369783223878504E-4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>33</v>
       </c>
       <c r="B24" s="1">
-        <v>0.108972267405539</v>
+        <v>8.4883882170655206E-2</v>
       </c>
       <c r="C24" s="1">
         <v>1.62396953112003</v>
@@ -1889,21 +1889,21 @@
         <v>-1.0787190975694701E-4</v>
       </c>
       <c r="F24" s="1">
-        <v>2.6521304066129399</v>
+        <v>2.5909093735917099</v>
       </c>
       <c r="G24" s="1">
-        <v>41.933413631928701</v>
+        <v>41.934661947052597</v>
       </c>
       <c r="H24" s="1">
-        <v>1.1289889289675E-3</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="42.75">
+        <v>1.1074301518603201E-3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B25" s="1">
-        <v>0.107940873985824</v>
+        <v>8.4153042797615304E-2</v>
       </c>
       <c r="C25" s="1">
         <v>1.6241066273141</v>
@@ -1915,16 +1915,16 @@
         <v>7.3904364256341599E-6</v>
       </c>
       <c r="F25" s="1">
-        <v>2.39688264160614</v>
+        <v>2.3357482344504699</v>
       </c>
       <c r="G25" s="1">
-        <v>39.964110004210902</v>
+        <v>40.953749600683999</v>
       </c>
       <c r="H25" s="1">
-        <v>6.36780711088425E-4</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
+        <v>7.5221203834955296E-4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -1934,7 +1934,7 @@
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
     </row>
-    <row r="27" spans="1:8">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -1944,7 +1944,7 @@
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
     </row>
-    <row r="28" spans="1:8">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -1954,7 +1954,7 @@
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
     </row>
-    <row r="29" spans="1:8">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -1964,7 +1964,7 @@
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
     </row>
-    <row r="30" spans="1:8">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -1974,7 +1974,7 @@
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
     </row>
-    <row r="31" spans="1:8">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -1984,7 +1984,7 @@
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -1994,7 +1994,7 @@
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
     </row>
-    <row r="33" spans="1:8">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -2004,7 +2004,7 @@
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
     </row>
-    <row r="34" spans="1:8">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -2021,10 +2021,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF8CB368-1F4F-4C65-B86B-93EC676CB77B}">
-  <dimension ref="A1:G34"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A1:M34"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2034,8 +2034,10 @@
       <c r="C1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="42.75">
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+    </row>
+    <row r="2" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -2043,7 +2045,7 @@
         <v>5.2401573655099698</v>
       </c>
       <c r="C2" s="1">
-        <v>0.10788210556906901</v>
+        <v>8.4020421663362793E-2</v>
       </c>
       <c r="F2">
         <v>894</v>
@@ -2051,8 +2053,10 @@
       <c r="G2">
         <v>456</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" ht="42.75">
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+    </row>
+    <row r="3" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -2060,7 +2064,7 @@
         <v>5.2402095305102501</v>
       </c>
       <c r="C3" s="1">
-        <v>0.107767689685955</v>
+        <v>8.3856539409502107E-2</v>
       </c>
       <c r="E3" t="s">
         <v>1</v>
@@ -2071,10 +2075,12 @@
       </c>
       <c r="G3">
         <f>AVERAGE(C2:C31)</f>
-        <v>0.10788639844759125</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="42.75">
+        <v>8.3990743181778446E-2</v>
+      </c>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+    </row>
+    <row r="4" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -2082,7 +2088,7 @@
         <v>5.2325481598897898</v>
       </c>
       <c r="C4" s="1">
-        <v>0.1085661885666</v>
+        <v>8.4441497497705006E-2</v>
       </c>
       <c r="E4" t="s">
         <v>2</v>
@@ -2093,10 +2099,12 @@
       </c>
       <c r="G4">
         <f>_xlfn.STDEV.S(C2:C32)</f>
-        <v>4.18616985875993E-4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="42.75">
+        <v>3.4221070261024404E-4</v>
+      </c>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+    </row>
+    <row r="5" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -2104,7 +2112,7 @@
         <v>5.2632048700287699</v>
       </c>
       <c r="C5" s="1">
-        <v>0.107813849166461</v>
+        <v>8.3922207540377103E-2</v>
       </c>
       <c r="E5" t="s">
         <v>3</v>
@@ -2115,10 +2123,12 @@
       </c>
       <c r="G5">
         <f>G4/G3/SQRT(COUNT(C2:C32))</f>
-        <v>7.9203528573635901E-4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="42.75">
+        <v>8.3168054613296123E-4</v>
+      </c>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+    </row>
+    <row r="6" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -2126,10 +2136,12 @@
         <v>5.2341542225512701</v>
       </c>
       <c r="C6" s="1">
-        <v>0.10768118552928301</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="42.75">
+        <v>8.3819979532311101E-2</v>
+      </c>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+    </row>
+    <row r="7" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
@@ -2137,10 +2149,12 @@
         <v>5.2499074678307798</v>
       </c>
       <c r="C7" s="1">
-        <v>0.10798815957236201</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="42.75">
+        <v>8.4065913892834104E-2</v>
+      </c>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+    </row>
+    <row r="8" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
@@ -2148,10 +2162,12 @@
         <v>5.2609478156281302</v>
       </c>
       <c r="C8" s="1">
-        <v>0.10796561723725399</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="42.75">
+        <v>8.4094869806041694E-2</v>
+      </c>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+    </row>
+    <row r="9" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
@@ -2159,10 +2175,12 @@
         <v>5.2522638411999596</v>
       </c>
       <c r="C9" s="1">
-        <v>0.107310696139959</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="42.75">
+        <v>8.3498425913598198E-2</v>
+      </c>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+    </row>
+    <row r="10" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
@@ -2170,10 +2188,12 @@
         <v>5.2381148673874796</v>
       </c>
       <c r="C10" s="1">
-        <v>0.107235378128852</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="42.75">
+        <v>8.3501392552088799E-2</v>
+      </c>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+    </row>
+    <row r="11" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
@@ -2181,10 +2201,12 @@
         <v>5.2236574261532196</v>
       </c>
       <c r="C11" s="1">
-        <v>0.107380313151722</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="42.75">
+        <v>8.3538886283743397E-2</v>
+      </c>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+    </row>
+    <row r="12" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
@@ -2192,10 +2214,12 @@
         <v>5.2262449444555799</v>
       </c>
       <c r="C12" s="1">
-        <v>0.107499657333732</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="42.75">
+        <v>8.3653316711863296E-2</v>
+      </c>
+      <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+    </row>
+    <row r="13" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>22</v>
       </c>
@@ -2203,10 +2227,12 @@
         <v>5.2457271314303799</v>
       </c>
       <c r="C13" s="1">
-        <v>0.107395325995434</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="42.75">
+        <v>8.36218907831483E-2</v>
+      </c>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+    </row>
+    <row r="14" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>23</v>
       </c>
@@ -2214,10 +2240,12 @@
         <v>5.2597760818477397</v>
       </c>
       <c r="C14" s="1">
-        <v>0.107617315330632</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="42.75">
+        <v>8.3768728051409405E-2</v>
+      </c>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+    </row>
+    <row r="15" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>24</v>
       </c>
@@ -2225,10 +2253,12 @@
         <v>5.2273625593786797</v>
       </c>
       <c r="C15" s="1">
-        <v>0.107631821742582</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="42.75">
+        <v>8.3798815283381206E-2</v>
+      </c>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+    </row>
+    <row r="16" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>25</v>
       </c>
@@ -2236,10 +2266,12 @@
         <v>5.2281725990355099</v>
       </c>
       <c r="C16" s="1">
-        <v>0.107773221003444</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="42.75">
+        <v>8.37952938220691E-2</v>
+      </c>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+    </row>
+    <row r="17" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>26</v>
       </c>
@@ -2247,10 +2279,12 @@
         <v>5.2464873820867899</v>
       </c>
       <c r="C17" s="1">
-        <v>0.108054680115061</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="42.75">
+        <v>8.4084000178888202E-2</v>
+      </c>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+    </row>
+    <row r="18" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>27</v>
       </c>
@@ -2258,10 +2292,12 @@
         <v>5.2357499987829099</v>
       </c>
       <c r="C18" s="1">
-        <v>0.108470442647848</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="42.75">
+        <v>8.4478909636109295E-2</v>
+      </c>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+    </row>
+    <row r="19" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>28</v>
       </c>
@@ -2269,10 +2305,12 @@
         <v>5.2426137496126399</v>
       </c>
       <c r="C19" s="1">
-        <v>0.108306765636387</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="42.75">
+        <v>8.4376066440544406E-2</v>
+      </c>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+    </row>
+    <row r="20" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>29</v>
       </c>
@@ -2280,10 +2318,12 @@
         <v>5.25389374708476</v>
       </c>
       <c r="C20" s="1">
-        <v>0.10817681982411</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="42.75">
+        <v>8.42642456111901E-2</v>
+      </c>
+      <c r="L20" s="1"/>
+      <c r="M20" s="1"/>
+    </row>
+    <row r="21" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>30</v>
       </c>
@@ -2291,10 +2331,12 @@
         <v>5.2452132048918996</v>
       </c>
       <c r="C21" s="1">
-        <v>0.107850584510117</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="42.75">
+        <v>8.3954508319290494E-2</v>
+      </c>
+      <c r="L21" s="1"/>
+      <c r="M21" s="1"/>
+    </row>
+    <row r="22" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>31</v>
       </c>
@@ -2302,10 +2344,12 @@
         <v>5.2477036957110901</v>
       </c>
       <c r="C22" s="1">
-        <v>0.108220094487482</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="42.75">
+        <v>8.4241621326531999E-2</v>
+      </c>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+    </row>
+    <row r="23" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>32</v>
       </c>
@@ -2313,10 +2357,12 @@
         <v>5.1912280334424699</v>
       </c>
       <c r="C23" s="1">
-        <v>0.107772509976481</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="42.75">
+        <v>8.39433811384213E-2</v>
+      </c>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+    </row>
+    <row r="24" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>33</v>
       </c>
@@ -2324,10 +2370,12 @@
         <v>5.2649162726060403</v>
       </c>
       <c r="C24" s="1">
-        <v>0.108972267405539</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="42.75">
+        <v>8.4883882170655206E-2</v>
+      </c>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+    </row>
+    <row r="25" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>34</v>
       </c>
@@ -2335,51 +2383,71 @@
         <v>5.2682959002266401</v>
       </c>
       <c r="C25" s="1">
-        <v>0.107940873985824</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3">
+        <v>8.4153042797615304E-2</v>
+      </c>
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
-    </row>
-    <row r="27" spans="1:3">
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
-    </row>
-    <row r="28" spans="1:3">
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
-    </row>
-    <row r="29" spans="1:3">
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
-    </row>
-    <row r="30" spans="1:3">
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
-    </row>
-    <row r="31" spans="1:3">
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
-    </row>
-    <row r="32" spans="1:3">
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
-    </row>
-    <row r="33" spans="1:3">
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
-    </row>
-    <row r="34" spans="1:3">
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="C34" s="1"/>
+      <c r="L34" s="1"/>
+      <c r="M34" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>